<commit_message>
Corrige rota /pedidos para suportar pedidos antigos (11 colunas) e novos (12 colunas), adiciona status padrão 'Recebido'
</commit_message>
<xml_diff>
--- a/pedidos.xlsx
+++ b/pedidos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,6 +527,11 @@
       <c r="K2" t="n">
         <v>165</v>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Pronto</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -582,6 +587,11 @@
       <c r="K3" t="n">
         <v>165</v>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Pronto</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -636,6 +646,411 @@
       </c>
       <c r="K4" t="n">
         <v>165</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Entregue</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>23/10/2026 21:34</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Daniel Tadaieski</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>48999443394</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Retirar no local</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Urussanga</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>dinheiro</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Big-American (X da casa) x1 (Subtotal R$279.00)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Calabresa x41</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>937</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>23/10/2026 21:34</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Daniel Tadaieski</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>48999443394</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Retirar no local</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Urussanga</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>dinheiro</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Big-American (X da casa) x1 (Subtotal R$279.00)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Calabresa x41</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>937</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>23/10/2026 21:34</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Daniel Tadaieski</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>48999443394</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Retirar no local</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Urussanga</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>dinheiro</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Big-American (X da casa) x1 (Subtotal R$279.00)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Calabresa x41</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>937</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>23/10/2026 21:34</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Daniel Tadaieski</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>48999443394</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Retirar no local</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Urussanga</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>dinheiro</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>X-Salada x1 (Subtotal R$23.00)</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>937</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>23/10/2026 21:34</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Daniel Tadaieski</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>48999443394</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Retirar no local</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Urussanga</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>dinheiro</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>X-Salada x1 (Subtotal R$23.00)</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>937</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>23/10/2026 21:34</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Daniel Tadaieski</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>48999443394</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Retirar no local</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Urussanga</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>dinheiro</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>X-Bacon x1 (Subtotal R$27.00)</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>937</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Entregue</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>23/10/2026 21:34</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Daniel Tadaieski</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>48999443394</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Retirar no local</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Urussanga</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>dinheiro</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>X-Bacon x1 (Subtotal R$27.00)</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>937</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Pronto</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Migrar pedidos para banco SQLite e ajustar rotas
</commit_message>
<xml_diff>
--- a/pedidos.xlsx
+++ b/pedidos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,21 +472,26 @@
           <t>Total</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23/10/2026 21:19</t>
+          <t>24/10/2026 09:09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DSSDSA</t>
+          <t>Daniel Tadaieski</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ADSDAS</t>
+          <t>48999443394</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -499,54 +504,42 @@
           <t>Urussanga</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>ASD</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>dinheiro</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ASD</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>X-Salada x1 (Subtotal R$55.00)</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Calabresa x3, Hambúrguer Extra x2</t>
-        </is>
-      </c>
+          <t>X-Salada x1 (Subtotal R$23.00)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>165</v>
+        <v>127</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Pronto</t>
+          <t>Recebido</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>23/10/2026 21:19</t>
+          <t>24/10/2026 09:09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DSSDSA</t>
+          <t>Daniel Tadaieski</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ADSDAS</t>
+          <t>48999443394</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -559,54 +552,42 @@
           <t>Urussanga</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>ASD</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>dinheiro</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>ASD</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>X-Salada x1 (Subtotal R$55.00)</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Calabresa x3, Hambúrguer Extra x2</t>
-        </is>
-      </c>
+          <t>X-Salada x1 (Subtotal R$23.00)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
-        <v>165</v>
+        <v>127</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Pronto</t>
+          <t>Recebido</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>23/10/2026 21:19</t>
+          <t>24/10/2026 09:09</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DSSDSA</t>
+          <t>Daniel Tadaieski</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ADSDAS</t>
+          <t>48999443394</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -619,44 +600,32 @@
           <t>Urussanga</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>ASD</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>dinheiro</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>ASD</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>X-Salada x1 (Subtotal R$55.00)</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Calabresa x3, Hambúrguer Extra x2</t>
-        </is>
-      </c>
+          <t>X-Bacon x1 (Subtotal R$27.00)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
-        <v>165</v>
+        <v>127</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Entregue</t>
+          <t>Recebido</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>23/10/2026 21:34</t>
+          <t>24/10/2026 09:09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -679,33 +648,21 @@
           <t>Urussanga</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>dinheiro</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>DSA</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Big-American (X da casa) x1 (Subtotal R$279.00)</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Calabresa x41</t>
-        </is>
-      </c>
+          <t>X-Bacon x1 (Subtotal R$27.00)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
-        <v>937</v>
+        <v>127</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -716,7 +673,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>23/10/2026 21:34</t>
+          <t>24/10/2026 09:09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -739,317 +696,25 @@
           <t>Urussanga</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>dinheiro</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>DSA</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Big-American (X da casa) x1 (Subtotal R$279.00)</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Calabresa x41</t>
-        </is>
-      </c>
+          <t>X-Bacon x1 (Subtotal R$27.00)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>937</v>
+        <v>127</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>Recebido</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>23/10/2026 21:34</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Daniel Tadaieski</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>48999443394</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Retirar no local</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Urussanga</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>dinheiro</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>DSA</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Big-American (X da casa) x1 (Subtotal R$279.00)</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Calabresa x41</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>937</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>23/10/2026 21:34</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Daniel Tadaieski</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>48999443394</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Retirar no local</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Urussanga</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>dinheiro</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>DSA</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>X-Salada x1 (Subtotal R$23.00)</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>937</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>23/10/2026 21:34</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Daniel Tadaieski</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>48999443394</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Retirar no local</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Urussanga</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>dinheiro</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>DSA</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>X-Salada x1 (Subtotal R$23.00)</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>937</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>23/10/2026 21:34</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Daniel Tadaieski</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>48999443394</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Retirar no local</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Urussanga</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>dinheiro</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>DSA</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>X-Bacon x1 (Subtotal R$27.00)</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>937</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Entregue</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>23/10/2026 21:34</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Daniel Tadaieski</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>48999443394</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Retirar no local</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Urussanga</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>dinheiro</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>DSA</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>X-Bacon x1 (Subtotal R$27.00)</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>937</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Pronto</t>
         </is>
       </c>
     </row>

</xml_diff>